<commit_message>
Strip new-item highlighting from check_reconstructed.xlsx
User: this is a distribution file, visual '[NEW]' markers dont belong
in it -- history should live in our own records (PROGRESS.md/
SESSION_LOG.md/git), not baked into the deliverable. Removed the
light-green fill and "[신규] YYYY-MM-DD 추가" remark text from all 7
rows that had accumulated it (1-4, 4-5, 5-7..5-11), matching each row
s fill/font to a normal (unhighlighted) row in the same sheet. Border
and other formatting were already uniform across rows and untouched.

Edited on rhel-prod per the DRM workflow (strip_new_markers.py, run
over ssh, deleted after use). Verified: no 00E2EFDA fill or 신규 text
remains anywhere in the workbook, fill_checklist.py still fills all
62 items correctly with no leftover highlighting in the output.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N4EYG9sknTPCcAMoGwekEs
</commit_message>
<xml_diff>
--- a/OV-Maintenance/check_reconstructed.xlsx
+++ b/OV-Maintenance/check_reconstructed.xlsx
@@ -875,32 +875,28 @@
       <c r="F4" s="7" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>1-4</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>VM 스케줄링 가능 Node의 kubevirt.io/schedulable 라벨을 확인한다.</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>oc get nodes -l kubevirt.io/schedulable=true</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>CNV 설치 대상 Worker/Infra 노드에 라벨이 정상 부여되어 있고 설계 노드 수와 일치</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr"/>
-      <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t>[신규] 2026-09-11 추가</t>
-        </is>
-      </c>
+      <c r="F5" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2222,33 +2218,29 @@
       <c r="F5" s="7" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>4-5</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Multus/OVN-Kubernetes 네트워크 플러그인 Pod 상태 확인</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>oc get pods -n openshift-multus
 oc get pods -n openshift-ovn-kubernetes</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>모든 Pod의 STATUS가 Running이고 RESTARTS가 비정상적으로 높지 않음</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr"/>
-      <c r="F6" s="9" t="inlineStr">
-        <is>
-          <t>[신규] 2026-09-11 추가</t>
-        </is>
-      </c>
+      <c r="F6" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2453,148 +2445,127 @@
       <c r="F7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>5-7</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>KubeVirt/CDI 플랫폼 컴포넌트 상태 확인 (HyperConverged CR, virt-*, cdi-* Pod)</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>oc get hco -n openshift-cnv
 oc get pods -n openshift-cnv -l kubevirt.io</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>HyperConverged AVAILABLE=True·DEGRADED=False, virt-operator/virt-controller/virt-handler/virt-api 및 cdi-* Pod 모두 Running</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr"/>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>[신규] 2026-09-11 추가</t>
-        </is>
-      </c>
+      <c r="F8" s="7" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>5-8</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>노드별 메모리 Capacity/Allocatable/Allocated(Request 소진율) 확인</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>oc describe node &lt;각 노드&gt;
 oc describe node &lt;각 노드&gt; | grep -A10 'Allocated resources'</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>Allocatable 대비 Allocated(Requests) 소진율이 과도하게 높지 않음 (오버커밋으로 인한 VM 스케줄링 실패 여지 확인)</t>
         </is>
       </c>
       <c r="E9" s="8" t="n"/>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>[신규] 2026-09-14 추가</t>
-        </is>
-      </c>
+      <c r="F9" s="7" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>5-9</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>OpenShift Virtualization 메모리 Overcommit(higherWorkloadDensity) 설정 확인</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>oc get hyperconverged kubevirt-hyperconverged -n openshift-cnv -o jsonpath={.spec.higherWorkloadDensity}</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>조직 정책과 일치하는 Overcommit 설정 값인지 확인 (미설정 시 기본 비활성)</t>
         </is>
       </c>
       <c r="E10" s="8" t="n"/>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>[신규] 2026-09-14 추가</t>
-        </is>
-      </c>
+      <c r="F10" s="7" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>5-10</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>전체 VM(virt-launcher) Pod의 memory request 확인</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>oc get pods -A -l kubevirt.io=virt-launcher -o custom-columns=NS:.metadata.namespace,NAME:.metadata.name,NODE:.spec.nodeName,REQ:.spec.containers[*].resources.requests.memory</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>각 VM(virt-launcher Pod)의 memory request가 설계값과 일치하고 특정 노드에 편중되지 않음</t>
         </is>
       </c>
       <c r="E11" s="8" t="n"/>
-      <c r="F11" s="9" t="inlineStr">
-        <is>
-          <t>[신규] 2026-09-14 추가</t>
-        </is>
-      </c>
+      <c r="F11" s="7" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>5-11</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>VM 스케줄링 실패(FailedScheduling) 이벤트 확인</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>oc get events -A --field-selector reason=FailedScheduling --sort-by=.lastTimestamp</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>FailedScheduling 이벤트 없음(있으면 사유를 확인해 request 소진/오버커밋 여부 판단)</t>
         </is>
       </c>
       <c r="E12" s="8" t="n"/>
-      <c r="F12" s="9" t="inlineStr">
-        <is>
-          <t>[신규] 2026-09-14 추가</t>
-        </is>
-      </c>
-    </row>
-    <row r="13"/>
+      <c r="F12" s="7" t="n"/>
+    </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
         <is>

</xml_diff>